<commit_message>
P2 mode facturation proprietaires et adresse David
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/02_TRAVAIL/Lot11_Controles/MASTER_CTRL_Coherence.xlsx
+++ b/02_TRAVAIL/Lot11_Controles/MASTER_CTRL_Coherence.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M52"/>
+  <dimension ref="A1:M51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -535,7 +535,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -586,7 +586,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -637,7 +637,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -739,7 +739,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -794,7 +794,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -853,7 +853,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -912,7 +912,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -971,7 +971,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -1030,7 +1030,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -1089,7 +1089,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -1148,7 +1148,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -1207,7 +1207,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -1266,7 +1266,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -1325,7 +1325,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -1384,7 +1384,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -1443,7 +1443,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -1502,7 +1502,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -1561,7 +1561,7 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -1620,7 +1620,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -1679,7 +1679,7 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -1734,7 +1734,7 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -1789,7 +1789,7 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -1844,7 +1844,7 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -1899,7 +1899,7 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -1954,7 +1954,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -2009,7 +2009,7 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -2064,7 +2064,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -2174,7 +2174,7 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2229,7 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -2284,7 +2284,7 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -2339,7 +2339,7 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -2394,7 +2394,7 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -2449,7 +2449,7 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -2504,7 +2504,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -2559,7 +2559,7 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -2614,7 +2614,7 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -2669,7 +2669,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -2724,7 +2724,7 @@
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -2779,7 +2779,7 @@
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -2834,7 +2834,7 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -2889,7 +2889,7 @@
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -2944,7 +2944,7 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -2995,7 +2995,7 @@
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -3046,7 +3046,7 @@
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -3097,43 +3097,51 @@
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>TRANSVERSE||MODE_FACTURATION_A_DEFINIR</t>
+          <t>2026-02||CLOTURE_IMPOSSIBLE_LIGNE_BANCAIRE_NON_CLASSEE</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>TRANSVERSE</t>
+          <t>BANQUE</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>REF_Proprietaires</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr"/>
+          <t>BANQUE_LOT8_IMPORT_REF_Cloture</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>2026-02</t>
+        </is>
+      </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>MODE_FACTURATION_A_DEFINIR</t>
+          <t>CLOTURE_IMPOSSIBLE_LIGNE_BANCAIRE_NON_CLASSEE</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>INFO</t>
+          <t>A_CONTROLER</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>12 proprietaires avec mode_facturation=A_DEFINIR. Bloquant pour Lot 12 (facturation). Non bloquant pour Lots 9-11.</t>
-        </is>
-      </c>
-      <c r="H49" t="inlineStr"/>
+          <t>Mois 2026-02 statut=OUVERT: 1 lignes RAPPROCHEMENT_REQUIS. Cloture impossible tant que rapprochements non resolus.</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>2026-02</t>
+        </is>
+      </c>
       <c r="I49" t="inlineStr"/>
       <c r="J49" t="inlineStr"/>
       <c r="K49" t="inlineStr">
@@ -3143,19 +3151,19 @@
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>Definir mode_facturation avant Lot 12.</t>
+          <t>Exporter donnees Airbnb et rapprocher RAPPROCH_AIRBNB_ATTENTE (Lot 8c).</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-02||CLOTURE_IMPOSSIBLE_LIGNE_BANCAIRE_NON_CLASSEE</t>
+          <t>2026-03||CLOTURE_IMPOSSIBLE_LIGNE_BANCAIRE_NON_CLASSEE</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -3170,7 +3178,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-03</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -3185,12 +3193,12 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Mois 2026-02 statut=OUVERT: 1 lignes RAPPROCHEMENT_REQUIS. Cloture impossible tant que rapprochements non resolus.</t>
+          <t>Mois 2026-03 statut=OUVERT: 31 lignes RAPPROCHEMENT_REQUIS. Cloture impossible tant que rapprochements non resolus.</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-03</t>
         </is>
       </c>
       <c r="I50" t="inlineStr"/>
@@ -3207,14 +3215,14 @@
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-03||CLOTURE_IMPOSSIBLE_LIGNE_BANCAIRE_NON_CLASSEE</t>
+          <t>2026-04||CLOTURE_IMPOSSIBLE_LIGNE_BANCAIRE_NON_CLASSEE</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -3229,7 +3237,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-04</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -3244,12 +3252,12 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Mois 2026-03 statut=OUVERT: 31 lignes RAPPROCHEMENT_REQUIS. Cloture impossible tant que rapprochements non resolus.</t>
+          <t>Mois 2026-04 statut=OUVERT: 20 lignes RAPPROCHEMENT_REQUIS. Cloture impossible tant que rapprochements non resolus.</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-04</t>
         </is>
       </c>
       <c r="I51" t="inlineStr"/>
@@ -3266,66 +3274,7 @@
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>2026-04||CLOTURE_IMPOSSIBLE_LIGNE_BANCAIRE_NON_CLASSEE</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>BANQUE</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>BANQUE_LOT8_IMPORT_REF_Cloture</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>2026-04</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>CLOTURE_IMPOSSIBLE_LIGNE_BANCAIRE_NON_CLASSEE</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t>Mois 2026-04 statut=OUVERT: 20 lignes RAPPROCHEMENT_REQUIS. Cloture impossible tant que rapprochements non resolus.</t>
-        </is>
-      </c>
-      <c r="H52" t="inlineStr">
-        <is>
-          <t>2026-04</t>
-        </is>
-      </c>
-      <c r="I52" t="inlineStr"/>
-      <c r="J52" t="inlineStr"/>
-      <c r="K52" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L52" t="inlineStr">
-        <is>
-          <t>Exporter donnees Airbnb et rapprocher RAPPROCH_AIRBNB_ATTENTE (Lot 8c).</t>
-        </is>
-      </c>
-      <c r="M52" t="inlineStr">
-        <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -3546,7 +3495,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -3605,7 +3554,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -3664,7 +3613,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -3723,7 +3672,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -3782,7 +3731,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -3841,7 +3790,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -3900,7 +3849,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -3959,7 +3908,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -4018,7 +3967,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -4077,7 +4026,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -4136,7 +4085,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -4195,7 +4144,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -4254,7 +4203,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -4313,7 +4262,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -4372,7 +4321,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -4427,7 +4376,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4431,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -4537,7 +4486,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -4592,7 +4541,7 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -4647,7 +4596,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -4702,7 +4651,7 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -4757,7 +4706,7 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -4812,7 +4761,7 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -4867,7 +4816,7 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -4922,7 +4871,7 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -4977,7 +4926,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -5032,7 +4981,7 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -5087,7 +5036,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -5142,7 +5091,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -5197,7 +5146,7 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -5252,7 +5201,7 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -5307,7 +5256,7 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -5362,7 +5311,7 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -5417,7 +5366,7 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -5472,7 +5421,7 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -5527,7 +5476,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -5582,7 +5531,7 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5586,7 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -5688,7 +5637,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -5739,7 +5688,7 @@
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -5790,7 +5739,7 @@
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -5849,7 +5798,7 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -5908,7 +5857,7 @@
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -5967,7 +5916,7 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -6148,7 +6097,7 @@
         <v>41</v>
       </c>
       <c r="D5" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Correctif Lot 11 - Resolution mappings listings
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/02_TRAVAIL/Lot11_Controles/MASTER_CTRL_Coherence.xlsx
+++ b/02_TRAVAIL/Lot11_Controles/MASTER_CTRL_Coherence.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M51"/>
+  <dimension ref="A1:M28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1686,27 +1686,23 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>nan||LISTING_ORPHELIN_A_CONTROLER</t>
+          <t>RESERVATIONS||VRBO_MONTANT_NON_RENSEIGNE</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>HOSTAWAY</t>
+          <t>RESERVATIONS</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>MASTER_CTRL_HA_Anomalies</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+          <t>MASTER_CALC_Reservations</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>LISTING_ORPHELIN_A_CONTROLER</t>
+          <t>VRBO_MONTANT_NON_RENSEIGNE</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1716,7 +1712,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Listing 515523 dans API Hostaway absent de REF_Logements</t>
+          <t>32 reservations HOSTAWAY_VRBO_A_CONTROLER sans montant valide. Saisie manuelle requise au Lot 4.</t>
         </is>
       </c>
       <c r="H23" t="inlineStr"/>
@@ -1729,7 +1725,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Resolution: ajouter listing au REF_Logements ou confirmer inactif.</t>
+          <t>Lots 4/4bis: saisir montants VRBO dans SAISIE_ReservationsHorsHostaway.xlsx</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -1741,27 +1737,23 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>60559486.0||LISTING_ORPHELIN_A_CONTROLER</t>
+          <t>COMMISSIONS||RESERVATION_A_CONTROLER_SANS_COMMISSION</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>HOSTAWAY</t>
+          <t>COMMISSIONS</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>MASTER_CTRL_HA_Anomalies</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>60559486.0</t>
-        </is>
-      </c>
+          <t>MASTER_CALC_Commissions</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>LISTING_ORPHELIN_A_CONTROLER</t>
+          <t>RESERVATION_A_CONTROLER_SANS_COMMISSION</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1771,7 +1763,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>listingMapId 556954 absent de REF_Logements — Lot 2 requis</t>
+          <t>59 reservations A_CONTROLER exclues du calcul automatique des commissions (VRBO + Direct). Net proprietaire incomplet pour ces 59 reservations.</t>
         </is>
       </c>
       <c r="H24" t="inlineStr"/>
@@ -1784,7 +1776,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>Resolution: ajouter listing au REF_Logements ou confirmer inactif.</t>
+          <t>Requiert saisie manuelle ou decision par reservation. Lots 4/4bis.</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -1796,27 +1788,23 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>58933140.0||LISTING_ORPHELIN_A_CONTROLER</t>
+          <t>MENAGES_EXT||MENAGE_EXTERNE_DATE_ABSENTE</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>HOSTAWAY</t>
+          <t>MENAGES_EXT</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>MASTER_CTRL_HA_Anomalies</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>58933140.0</t>
-        </is>
-      </c>
+          <t>MASTER_FACT_MEN_MenagesExternes</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>LISTING_ORPHELIN_A_CONTROLER</t>
+          <t>MENAGE_EXTERNE_DATE_ABSENTE</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1826,7 +1814,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>listingMapId 515523 absent de REF_Logements — Lot 2 requis</t>
+          <t>9 lignes menages externes sans date_menage precise. Exclues de VUE_ACTIVE.</t>
         </is>
       </c>
       <c r="H25" t="inlineStr"/>
@@ -1839,7 +1827,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>Resolution: ajouter listing au REF_Logements ou confirmer inactif.</t>
+          <t>Precision date requise aupres du prestataire (Aissata fac.2026-37).</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
@@ -1851,27 +1839,27 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>58765312.0||LISTING_ORPHELIN_A_CONTROLER</t>
+          <t>2026-02||CLOTURE_IMPOSSIBLE_LIGNE_BANCAIRE_NON_CLASSEE</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>HOSTAWAY</t>
+          <t>BANQUE</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>MASTER_CTRL_HA_Anomalies</t>
+          <t>BANQUE_LOT8_IMPORT_REF_Cloture</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>58765312.0</t>
+          <t>2026-02</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>LISTING_ORPHELIN_A_CONTROLER</t>
+          <t>CLOTURE_IMPOSSIBLE_LIGNE_BANCAIRE_NON_CLASSEE</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1881,10 +1869,14 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>listingMapId 515523 absent de REF_Logements — Lot 2 requis</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr"/>
+          <t>Mois 2026-02 statut=OUVERT: 1 lignes RAPPROCHEMENT_REQUIS. Cloture impossible tant que rapprochements non resolus.</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>2026-02</t>
+        </is>
+      </c>
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr">
@@ -1894,7 +1886,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>Resolution: ajouter listing au REF_Logements ou confirmer inactif.</t>
+          <t>Exporter donnees Airbnb et rapprocher RAPPROCH_AIRBNB_ATTENTE (Lot 8c).</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -1906,27 +1898,27 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>58607186.0||LISTING_ORPHELIN_A_CONTROLER</t>
+          <t>2026-03||CLOTURE_IMPOSSIBLE_LIGNE_BANCAIRE_NON_CLASSEE</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>HOSTAWAY</t>
+          <t>BANQUE</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>MASTER_CTRL_HA_Anomalies</t>
+          <t>BANQUE_LOT8_IMPORT_REF_Cloture</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>58607186.0</t>
+          <t>2026-03</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>LISTING_ORPHELIN_A_CONTROLER</t>
+          <t>CLOTURE_IMPOSSIBLE_LIGNE_BANCAIRE_NON_CLASSEE</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1936,10 +1928,14 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>listingMapId 515523 absent de REF_Logements — Lot 2 requis</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr"/>
+          <t>Mois 2026-03 statut=OUVERT: 31 lignes RAPPROCHEMENT_REQUIS. Cloture impossible tant que rapprochements non resolus.</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr">
@@ -1949,7 +1945,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>Resolution: ajouter listing au REF_Logements ou confirmer inactif.</t>
+          <t>Exporter donnees Airbnb et rapprocher RAPPROCH_AIRBNB_ATTENTE (Lot 8c).</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -1961,27 +1957,27 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>58607180.0||LISTING_ORPHELIN_A_CONTROLER</t>
+          <t>2026-04||CLOTURE_IMPOSSIBLE_LIGNE_BANCAIRE_NON_CLASSEE</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>HOSTAWAY</t>
+          <t>BANQUE</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>MASTER_CTRL_HA_Anomalies</t>
+          <t>BANQUE_LOT8_IMPORT_REF_Cloture</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>58607180.0</t>
+          <t>2026-04</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>LISTING_ORPHELIN_A_CONTROLER</t>
+          <t>CLOTURE_IMPOSSIBLE_LIGNE_BANCAIRE_NON_CLASSEE</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1991,10 +1987,14 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>listingMapId 515523 absent de REF_Logements — Lot 2 requis</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr"/>
+          <t>Mois 2026-04 statut=OUVERT: 20 lignes RAPPROCHEMENT_REQUIS. Cloture impossible tant que rapprochements non resolus.</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr">
@@ -2004,1275 +2004,10 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>Resolution: ajouter listing au REF_Logements ou confirmer inactif.</t>
+          <t>Exporter donnees Airbnb et rapprocher RAPPROCH_AIRBNB_ATTENTE (Lot 8c).</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>58607170.0||LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>HOSTAWAY</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>MASTER_CTRL_HA_Anomalies</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>58607170.0</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>listingMapId 515523 absent de REF_Logements — Lot 2 requis</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L29" t="inlineStr">
-        <is>
-          <t>Resolution: ajouter listing au REF_Logements ou confirmer inactif.</t>
-        </is>
-      </c>
-      <c r="M29" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>58607164.0||LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>HOSTAWAY</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>MASTER_CTRL_HA_Anomalies</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>58607164.0</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>listingMapId 515523 absent de REF_Logements — Lot 2 requis</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L30" t="inlineStr">
-        <is>
-          <t>Resolution: ajouter listing au REF_Logements ou confirmer inactif.</t>
-        </is>
-      </c>
-      <c r="M30" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>58607160.0||LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>HOSTAWAY</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>MASTER_CTRL_HA_Anomalies</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>58607160.0</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>listingMapId 515523 absent de REF_Logements — Lot 2 requis</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L31" t="inlineStr">
-        <is>
-          <t>Resolution: ajouter listing au REF_Logements ou confirmer inactif.</t>
-        </is>
-      </c>
-      <c r="M31" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>58607154.0||LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>HOSTAWAY</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>MASTER_CTRL_HA_Anomalies</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>58607154.0</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>listingMapId 515523 absent de REF_Logements — Lot 2 requis</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L32" t="inlineStr">
-        <is>
-          <t>Resolution: ajouter listing au REF_Logements ou confirmer inactif.</t>
-        </is>
-      </c>
-      <c r="M32" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>58607149.0||LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>HOSTAWAY</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>MASTER_CTRL_HA_Anomalies</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>58607149.0</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>listingMapId 515523 absent de REF_Logements — Lot 2 requis</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L33" t="inlineStr">
-        <is>
-          <t>Resolution: ajouter listing au REF_Logements ou confirmer inactif.</t>
-        </is>
-      </c>
-      <c r="M33" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>58607145.0||LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>HOSTAWAY</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>MASTER_CTRL_HA_Anomalies</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>58607145.0</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>listingMapId 515523 absent de REF_Logements — Lot 2 requis</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L34" t="inlineStr">
-        <is>
-          <t>Resolution: ajouter listing au REF_Logements ou confirmer inactif.</t>
-        </is>
-      </c>
-      <c r="M34" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>58607138.0||LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>HOSTAWAY</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>MASTER_CTRL_HA_Anomalies</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>58607138.0</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>listingMapId 515523 absent de REF_Logements — Lot 2 requis</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L35" t="inlineStr">
-        <is>
-          <t>Resolution: ajouter listing au REF_Logements ou confirmer inactif.</t>
-        </is>
-      </c>
-      <c r="M35" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>58607127.0||LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>HOSTAWAY</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>MASTER_CTRL_HA_Anomalies</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>58607127.0</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>listingMapId 515523 absent de REF_Logements — Lot 2 requis</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L36" t="inlineStr">
-        <is>
-          <t>Resolution: ajouter listing au REF_Logements ou confirmer inactif.</t>
-        </is>
-      </c>
-      <c r="M36" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>58607119.0||LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>HOSTAWAY</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>MASTER_CTRL_HA_Anomalies</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>58607119.0</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>listingMapId 515523 absent de REF_Logements — Lot 2 requis</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L37" t="inlineStr">
-        <is>
-          <t>Resolution: ajouter listing au REF_Logements ou confirmer inactif.</t>
-        </is>
-      </c>
-      <c r="M37" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>58607115.0||LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>HOSTAWAY</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>MASTER_CTRL_HA_Anomalies</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>58607115.0</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>listingMapId 515523 absent de REF_Logements — Lot 2 requis</t>
-        </is>
-      </c>
-      <c r="H38" t="inlineStr"/>
-      <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L38" t="inlineStr">
-        <is>
-          <t>Resolution: ajouter listing au REF_Logements ou confirmer inactif.</t>
-        </is>
-      </c>
-      <c r="M38" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>58607112.0||LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>HOSTAWAY</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>MASTER_CTRL_HA_Anomalies</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>58607112.0</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>listingMapId 515523 absent de REF_Logements — Lot 2 requis</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr"/>
-      <c r="I39" t="inlineStr"/>
-      <c r="J39" t="inlineStr"/>
-      <c r="K39" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L39" t="inlineStr">
-        <is>
-          <t>Resolution: ajouter listing au REF_Logements ou confirmer inactif.</t>
-        </is>
-      </c>
-      <c r="M39" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>58607111.0||LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>HOSTAWAY</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>MASTER_CTRL_HA_Anomalies</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>58607111.0</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>listingMapId 515523 absent de REF_Logements — Lot 2 requis</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr"/>
-      <c r="K40" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L40" t="inlineStr">
-        <is>
-          <t>Resolution: ajouter listing au REF_Logements ou confirmer inactif.</t>
-        </is>
-      </c>
-      <c r="M40" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>58607108.0||LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>HOSTAWAY</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>MASTER_CTRL_HA_Anomalies</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>58607108.0</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>listingMapId 515523 absent de REF_Logements — Lot 2 requis</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr"/>
-      <c r="K41" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L41" t="inlineStr">
-        <is>
-          <t>Resolution: ajouter listing au REF_Logements ou confirmer inactif.</t>
-        </is>
-      </c>
-      <c r="M41" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>58607104.0||LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>HOSTAWAY</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>MASTER_CTRL_HA_Anomalies</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>58607104.0</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>listingMapId 515523 absent de REF_Logements — Lot 2 requis</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr"/>
-      <c r="I42" t="inlineStr"/>
-      <c r="J42" t="inlineStr"/>
-      <c r="K42" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L42" t="inlineStr">
-        <is>
-          <t>Resolution: ajouter listing au REF_Logements ou confirmer inactif.</t>
-        </is>
-      </c>
-      <c r="M42" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>58607096.0||LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>HOSTAWAY</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>MASTER_CTRL_HA_Anomalies</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>58607096.0</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>listingMapId 515523 absent de REF_Logements — Lot 2 requis</t>
-        </is>
-      </c>
-      <c r="H43" t="inlineStr"/>
-      <c r="I43" t="inlineStr"/>
-      <c r="J43" t="inlineStr"/>
-      <c r="K43" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L43" t="inlineStr">
-        <is>
-          <t>Resolution: ajouter listing au REF_Logements ou confirmer inactif.</t>
-        </is>
-      </c>
-      <c r="M43" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>58606195.0||LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>HOSTAWAY</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>MASTER_CTRL_HA_Anomalies</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>58606195.0</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>listingMapId 515523 absent de REF_Logements — Lot 2 requis</t>
-        </is>
-      </c>
-      <c r="H44" t="inlineStr"/>
-      <c r="I44" t="inlineStr"/>
-      <c r="J44" t="inlineStr"/>
-      <c r="K44" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L44" t="inlineStr">
-        <is>
-          <t>Resolution: ajouter listing au REF_Logements ou confirmer inactif.</t>
-        </is>
-      </c>
-      <c r="M44" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>58606185.0||LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>HOSTAWAY</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>MASTER_CTRL_HA_Anomalies</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>58606185.0</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>listingMapId 515523 absent de REF_Logements — Lot 2 requis</t>
-        </is>
-      </c>
-      <c r="H45" t="inlineStr"/>
-      <c r="I45" t="inlineStr"/>
-      <c r="J45" t="inlineStr"/>
-      <c r="K45" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L45" t="inlineStr">
-        <is>
-          <t>Resolution: ajouter listing au REF_Logements ou confirmer inactif.</t>
-        </is>
-      </c>
-      <c r="M45" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>RESERVATIONS||VRBO_MONTANT_NON_RENSEIGNE</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>RESERVATIONS</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>MASTER_CALC_Reservations</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr"/>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>VRBO_MONTANT_NON_RENSEIGNE</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>32 reservations HOSTAWAY_VRBO_A_CONTROLER sans montant valide. Saisie manuelle requise au Lot 4.</t>
-        </is>
-      </c>
-      <c r="H46" t="inlineStr"/>
-      <c r="I46" t="inlineStr"/>
-      <c r="J46" t="inlineStr"/>
-      <c r="K46" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L46" t="inlineStr">
-        <is>
-          <t>Lots 4/4bis: saisir montants VRBO dans SAISIE_ReservationsHorsHostaway.xlsx</t>
-        </is>
-      </c>
-      <c r="M46" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>COMMISSIONS||RESERVATION_A_CONTROLER_SANS_COMMISSION</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>COMMISSIONS</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>MASTER_CALC_Commissions</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr"/>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>RESERVATION_A_CONTROLER_SANS_COMMISSION</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>59 reservations A_CONTROLER exclues du calcul automatique des commissions (VRBO + Direct). Net proprietaire incomplet pour ces 59 reservations.</t>
-        </is>
-      </c>
-      <c r="H47" t="inlineStr"/>
-      <c r="I47" t="inlineStr"/>
-      <c r="J47" t="inlineStr"/>
-      <c r="K47" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L47" t="inlineStr">
-        <is>
-          <t>Requiert saisie manuelle ou decision par reservation. Lots 4/4bis.</t>
-        </is>
-      </c>
-      <c r="M47" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>MENAGES_EXT||MENAGE_EXTERNE_DATE_ABSENTE</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>MENAGES_EXT</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>MASTER_FACT_MEN_MenagesExternes</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr"/>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>MENAGE_EXTERNE_DATE_ABSENTE</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>9 lignes menages externes sans date_menage precise. Exclues de VUE_ACTIVE.</t>
-        </is>
-      </c>
-      <c r="H48" t="inlineStr"/>
-      <c r="I48" t="inlineStr"/>
-      <c r="J48" t="inlineStr"/>
-      <c r="K48" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L48" t="inlineStr">
-        <is>
-          <t>Precision date requise aupres du prestataire (Aissata fac.2026-37).</t>
-        </is>
-      </c>
-      <c r="M48" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>2026-02||CLOTURE_IMPOSSIBLE_LIGNE_BANCAIRE_NON_CLASSEE</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>BANQUE</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>BANQUE_LOT8_IMPORT_REF_Cloture</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>2026-02</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>CLOTURE_IMPOSSIBLE_LIGNE_BANCAIRE_NON_CLASSEE</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>Mois 2026-02 statut=OUVERT: 1 lignes RAPPROCHEMENT_REQUIS. Cloture impossible tant que rapprochements non resolus.</t>
-        </is>
-      </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>2026-02</t>
-        </is>
-      </c>
-      <c r="I49" t="inlineStr"/>
-      <c r="J49" t="inlineStr"/>
-      <c r="K49" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L49" t="inlineStr">
-        <is>
-          <t>Exporter donnees Airbnb et rapprocher RAPPROCH_AIRBNB_ATTENTE (Lot 8c).</t>
-        </is>
-      </c>
-      <c r="M49" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>2026-03||CLOTURE_IMPOSSIBLE_LIGNE_BANCAIRE_NON_CLASSEE</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>BANQUE</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>BANQUE_LOT8_IMPORT_REF_Cloture</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>2026-03</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>CLOTURE_IMPOSSIBLE_LIGNE_BANCAIRE_NON_CLASSEE</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>Mois 2026-03 statut=OUVERT: 31 lignes RAPPROCHEMENT_REQUIS. Cloture impossible tant que rapprochements non resolus.</t>
-        </is>
-      </c>
-      <c r="H50" t="inlineStr">
-        <is>
-          <t>2026-03</t>
-        </is>
-      </c>
-      <c r="I50" t="inlineStr"/>
-      <c r="J50" t="inlineStr"/>
-      <c r="K50" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L50" t="inlineStr">
-        <is>
-          <t>Exporter donnees Airbnb et rapprocher RAPPROCH_AIRBNB_ATTENTE (Lot 8c).</t>
-        </is>
-      </c>
-      <c r="M50" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>2026-04||CLOTURE_IMPOSSIBLE_LIGNE_BANCAIRE_NON_CLASSEE</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>BANQUE</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>BANQUE_LOT8_IMPORT_REF_Cloture</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>2026-04</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>CLOTURE_IMPOSSIBLE_LIGNE_BANCAIRE_NON_CLASSEE</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G51" t="inlineStr">
-        <is>
-          <t>Mois 2026-04 statut=OUVERT: 20 lignes RAPPROCHEMENT_REQUIS. Cloture impossible tant que rapprochements non resolus.</t>
-        </is>
-      </c>
-      <c r="H51" t="inlineStr">
-        <is>
-          <t>2026-04</t>
-        </is>
-      </c>
-      <c r="I51" t="inlineStr"/>
-      <c r="J51" t="inlineStr"/>
-      <c r="K51" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L51" t="inlineStr">
-        <is>
-          <t>Exporter donnees Airbnb et rapprocher RAPPROCH_AIRBNB_ATTENTE (Lot 8c).</t>
-        </is>
-      </c>
-      <c r="M51" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
@@ -3370,7 +2105,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M45"/>
+  <dimension ref="A1:M22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4328,27 +3063,23 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>nan||LISTING_ORPHELIN_A_CONTROLER</t>
+          <t>RESERVATIONS||VRBO_MONTANT_NON_RENSEIGNE</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>HOSTAWAY</t>
+          <t>RESERVATIONS</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>MASTER_CTRL_HA_Anomalies</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+          <t>MASTER_CALC_Reservations</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>LISTING_ORPHELIN_A_CONTROLER</t>
+          <t>VRBO_MONTANT_NON_RENSEIGNE</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -4358,7 +3089,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Listing 515523 dans API Hostaway absent de REF_Logements</t>
+          <t>32 reservations HOSTAWAY_VRBO_A_CONTROLER sans montant valide. Saisie manuelle requise au Lot 4.</t>
         </is>
       </c>
       <c r="H17" t="inlineStr"/>
@@ -4371,7 +3102,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>Resolution: ajouter listing au REF_Logements ou confirmer inactif.</t>
+          <t>Lots 4/4bis: saisir montants VRBO dans SAISIE_ReservationsHorsHostaway.xlsx</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -4383,27 +3114,23 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>60559486.0||LISTING_ORPHELIN_A_CONTROLER</t>
+          <t>COMMISSIONS||RESERVATION_A_CONTROLER_SANS_COMMISSION</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>HOSTAWAY</t>
+          <t>COMMISSIONS</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>MASTER_CTRL_HA_Anomalies</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>60559486.0</t>
-        </is>
-      </c>
+          <t>MASTER_CALC_Commissions</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>LISTING_ORPHELIN_A_CONTROLER</t>
+          <t>RESERVATION_A_CONTROLER_SANS_COMMISSION</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -4413,7 +3140,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>listingMapId 556954 absent de REF_Logements — Lot 2 requis</t>
+          <t>59 reservations A_CONTROLER exclues du calcul automatique des commissions (VRBO + Direct). Net proprietaire incomplet pour ces 59 reservations.</t>
         </is>
       </c>
       <c r="H18" t="inlineStr"/>
@@ -4426,7 +3153,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>Resolution: ajouter listing au REF_Logements ou confirmer inactif.</t>
+          <t>Requiert saisie manuelle ou decision par reservation. Lots 4/4bis.</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -4438,27 +3165,23 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>58933140.0||LISTING_ORPHELIN_A_CONTROLER</t>
+          <t>MENAGES_EXT||MENAGE_EXTERNE_DATE_ABSENTE</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>HOSTAWAY</t>
+          <t>MENAGES_EXT</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>MASTER_CTRL_HA_Anomalies</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>58933140.0</t>
-        </is>
-      </c>
+          <t>MASTER_FACT_MEN_MenagesExternes</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>LISTING_ORPHELIN_A_CONTROLER</t>
+          <t>MENAGE_EXTERNE_DATE_ABSENTE</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -4468,7 +3191,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>listingMapId 515523 absent de REF_Logements — Lot 2 requis</t>
+          <t>9 lignes menages externes sans date_menage precise. Exclues de VUE_ACTIVE.</t>
         </is>
       </c>
       <c r="H19" t="inlineStr"/>
@@ -4481,7 +3204,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>Resolution: ajouter listing au REF_Logements ou confirmer inactif.</t>
+          <t>Precision date requise aupres du prestataire (Aissata fac.2026-37).</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -4493,27 +3216,27 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>58765312.0||LISTING_ORPHELIN_A_CONTROLER</t>
+          <t>2026-02||CLOTURE_IMPOSSIBLE_LIGNE_BANCAIRE_NON_CLASSEE</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>HOSTAWAY</t>
+          <t>BANQUE</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>MASTER_CTRL_HA_Anomalies</t>
+          <t>BANQUE_LOT8_IMPORT_REF_Cloture</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>58765312.0</t>
+          <t>2026-02</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>LISTING_ORPHELIN_A_CONTROLER</t>
+          <t>CLOTURE_IMPOSSIBLE_LIGNE_BANCAIRE_NON_CLASSEE</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -4523,10 +3246,14 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>listingMapId 515523 absent de REF_Logements — Lot 2 requis</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr"/>
+          <t>Mois 2026-02 statut=OUVERT: 1 lignes RAPPROCHEMENT_REQUIS. Cloture impossible tant que rapprochements non resolus.</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>2026-02</t>
+        </is>
+      </c>
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr">
@@ -4536,7 +3263,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Resolution: ajouter listing au REF_Logements ou confirmer inactif.</t>
+          <t>Exporter donnees Airbnb et rapprocher RAPPROCH_AIRBNB_ATTENTE (Lot 8c).</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -4548,27 +3275,27 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>58607186.0||LISTING_ORPHELIN_A_CONTROLER</t>
+          <t>2026-03||CLOTURE_IMPOSSIBLE_LIGNE_BANCAIRE_NON_CLASSEE</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>HOSTAWAY</t>
+          <t>BANQUE</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>MASTER_CTRL_HA_Anomalies</t>
+          <t>BANQUE_LOT8_IMPORT_REF_Cloture</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>58607186.0</t>
+          <t>2026-03</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>LISTING_ORPHELIN_A_CONTROLER</t>
+          <t>CLOTURE_IMPOSSIBLE_LIGNE_BANCAIRE_NON_CLASSEE</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -4578,10 +3305,14 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>listingMapId 515523 absent de REF_Logements — Lot 2 requis</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr"/>
+          <t>Mois 2026-03 statut=OUVERT: 31 lignes RAPPROCHEMENT_REQUIS. Cloture impossible tant que rapprochements non resolus.</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr">
@@ -4591,7 +3322,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>Resolution: ajouter listing au REF_Logements ou confirmer inactif.</t>
+          <t>Exporter donnees Airbnb et rapprocher RAPPROCH_AIRBNB_ATTENTE (Lot 8c).</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -4603,27 +3334,27 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>58607180.0||LISTING_ORPHELIN_A_CONTROLER</t>
+          <t>2026-04||CLOTURE_IMPOSSIBLE_LIGNE_BANCAIRE_NON_CLASSEE</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>HOSTAWAY</t>
+          <t>BANQUE</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>MASTER_CTRL_HA_Anomalies</t>
+          <t>BANQUE_LOT8_IMPORT_REF_Cloture</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>58607180.0</t>
+          <t>2026-04</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>LISTING_ORPHELIN_A_CONTROLER</t>
+          <t>CLOTURE_IMPOSSIBLE_LIGNE_BANCAIRE_NON_CLASSEE</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -4633,10 +3364,14 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>listingMapId 515523 absent de REF_Logements — Lot 2 requis</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr"/>
+          <t>Mois 2026-04 statut=OUVERT: 20 lignes RAPPROCHEMENT_REQUIS. Cloture impossible tant que rapprochements non resolus.</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr">
@@ -4646,1275 +3381,10 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>Resolution: ajouter listing au REF_Logements ou confirmer inactif.</t>
+          <t>Exporter donnees Airbnb et rapprocher RAPPROCH_AIRBNB_ATTENTE (Lot 8c).</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>58607170.0||LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>HOSTAWAY</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>MASTER_CTRL_HA_Anomalies</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>58607170.0</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>listingMapId 515523 absent de REF_Logements — Lot 2 requis</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t>Resolution: ajouter listing au REF_Logements ou confirmer inactif.</t>
-        </is>
-      </c>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>58607164.0||LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>HOSTAWAY</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>MASTER_CTRL_HA_Anomalies</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>58607164.0</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>listingMapId 515523 absent de REF_Logements — Lot 2 requis</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L24" t="inlineStr">
-        <is>
-          <t>Resolution: ajouter listing au REF_Logements ou confirmer inactif.</t>
-        </is>
-      </c>
-      <c r="M24" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>58607160.0||LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>HOSTAWAY</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>MASTER_CTRL_HA_Anomalies</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>58607160.0</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>listingMapId 515523 absent de REF_Logements — Lot 2 requis</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L25" t="inlineStr">
-        <is>
-          <t>Resolution: ajouter listing au REF_Logements ou confirmer inactif.</t>
-        </is>
-      </c>
-      <c r="M25" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>58607154.0||LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>HOSTAWAY</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>MASTER_CTRL_HA_Anomalies</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>58607154.0</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>listingMapId 515523 absent de REF_Logements — Lot 2 requis</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L26" t="inlineStr">
-        <is>
-          <t>Resolution: ajouter listing au REF_Logements ou confirmer inactif.</t>
-        </is>
-      </c>
-      <c r="M26" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>58607149.0||LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>HOSTAWAY</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>MASTER_CTRL_HA_Anomalies</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>58607149.0</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>listingMapId 515523 absent de REF_Logements — Lot 2 requis</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L27" t="inlineStr">
-        <is>
-          <t>Resolution: ajouter listing au REF_Logements ou confirmer inactif.</t>
-        </is>
-      </c>
-      <c r="M27" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>58607145.0||LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>HOSTAWAY</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>MASTER_CTRL_HA_Anomalies</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>58607145.0</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>listingMapId 515523 absent de REF_Logements — Lot 2 requis</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L28" t="inlineStr">
-        <is>
-          <t>Resolution: ajouter listing au REF_Logements ou confirmer inactif.</t>
-        </is>
-      </c>
-      <c r="M28" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>58607138.0||LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>HOSTAWAY</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>MASTER_CTRL_HA_Anomalies</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>58607138.0</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>listingMapId 515523 absent de REF_Logements — Lot 2 requis</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L29" t="inlineStr">
-        <is>
-          <t>Resolution: ajouter listing au REF_Logements ou confirmer inactif.</t>
-        </is>
-      </c>
-      <c r="M29" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>58607127.0||LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>HOSTAWAY</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>MASTER_CTRL_HA_Anomalies</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>58607127.0</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>listingMapId 515523 absent de REF_Logements — Lot 2 requis</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L30" t="inlineStr">
-        <is>
-          <t>Resolution: ajouter listing au REF_Logements ou confirmer inactif.</t>
-        </is>
-      </c>
-      <c r="M30" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>58607119.0||LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>HOSTAWAY</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>MASTER_CTRL_HA_Anomalies</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>58607119.0</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>listingMapId 515523 absent de REF_Logements — Lot 2 requis</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L31" t="inlineStr">
-        <is>
-          <t>Resolution: ajouter listing au REF_Logements ou confirmer inactif.</t>
-        </is>
-      </c>
-      <c r="M31" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>58607115.0||LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>HOSTAWAY</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>MASTER_CTRL_HA_Anomalies</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>58607115.0</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>listingMapId 515523 absent de REF_Logements — Lot 2 requis</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L32" t="inlineStr">
-        <is>
-          <t>Resolution: ajouter listing au REF_Logements ou confirmer inactif.</t>
-        </is>
-      </c>
-      <c r="M32" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>58607112.0||LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>HOSTAWAY</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>MASTER_CTRL_HA_Anomalies</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>58607112.0</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>listingMapId 515523 absent de REF_Logements — Lot 2 requis</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L33" t="inlineStr">
-        <is>
-          <t>Resolution: ajouter listing au REF_Logements ou confirmer inactif.</t>
-        </is>
-      </c>
-      <c r="M33" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>58607111.0||LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>HOSTAWAY</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>MASTER_CTRL_HA_Anomalies</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>58607111.0</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>listingMapId 515523 absent de REF_Logements — Lot 2 requis</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L34" t="inlineStr">
-        <is>
-          <t>Resolution: ajouter listing au REF_Logements ou confirmer inactif.</t>
-        </is>
-      </c>
-      <c r="M34" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>58607108.0||LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>HOSTAWAY</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>MASTER_CTRL_HA_Anomalies</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>58607108.0</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>listingMapId 515523 absent de REF_Logements — Lot 2 requis</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L35" t="inlineStr">
-        <is>
-          <t>Resolution: ajouter listing au REF_Logements ou confirmer inactif.</t>
-        </is>
-      </c>
-      <c r="M35" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>58607104.0||LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>HOSTAWAY</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>MASTER_CTRL_HA_Anomalies</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>58607104.0</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>listingMapId 515523 absent de REF_Logements — Lot 2 requis</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L36" t="inlineStr">
-        <is>
-          <t>Resolution: ajouter listing au REF_Logements ou confirmer inactif.</t>
-        </is>
-      </c>
-      <c r="M36" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>58607096.0||LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>HOSTAWAY</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>MASTER_CTRL_HA_Anomalies</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>58607096.0</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>listingMapId 515523 absent de REF_Logements — Lot 2 requis</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L37" t="inlineStr">
-        <is>
-          <t>Resolution: ajouter listing au REF_Logements ou confirmer inactif.</t>
-        </is>
-      </c>
-      <c r="M37" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>58606195.0||LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>HOSTAWAY</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>MASTER_CTRL_HA_Anomalies</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>58606195.0</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>listingMapId 515523 absent de REF_Logements — Lot 2 requis</t>
-        </is>
-      </c>
-      <c r="H38" t="inlineStr"/>
-      <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L38" t="inlineStr">
-        <is>
-          <t>Resolution: ajouter listing au REF_Logements ou confirmer inactif.</t>
-        </is>
-      </c>
-      <c r="M38" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>58606185.0||LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>HOSTAWAY</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>MASTER_CTRL_HA_Anomalies</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>58606185.0</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>LISTING_ORPHELIN_A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>listingMapId 515523 absent de REF_Logements — Lot 2 requis</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr"/>
-      <c r="I39" t="inlineStr"/>
-      <c r="J39" t="inlineStr"/>
-      <c r="K39" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L39" t="inlineStr">
-        <is>
-          <t>Resolution: ajouter listing au REF_Logements ou confirmer inactif.</t>
-        </is>
-      </c>
-      <c r="M39" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>RESERVATIONS||VRBO_MONTANT_NON_RENSEIGNE</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>RESERVATIONS</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>MASTER_CALC_Reservations</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr"/>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>VRBO_MONTANT_NON_RENSEIGNE</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>32 reservations HOSTAWAY_VRBO_A_CONTROLER sans montant valide. Saisie manuelle requise au Lot 4.</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr"/>
-      <c r="K40" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L40" t="inlineStr">
-        <is>
-          <t>Lots 4/4bis: saisir montants VRBO dans SAISIE_ReservationsHorsHostaway.xlsx</t>
-        </is>
-      </c>
-      <c r="M40" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>COMMISSIONS||RESERVATION_A_CONTROLER_SANS_COMMISSION</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>COMMISSIONS</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>MASTER_CALC_Commissions</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr"/>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>RESERVATION_A_CONTROLER_SANS_COMMISSION</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>59 reservations A_CONTROLER exclues du calcul automatique des commissions (VRBO + Direct). Net proprietaire incomplet pour ces 59 reservations.</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr"/>
-      <c r="K41" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L41" t="inlineStr">
-        <is>
-          <t>Requiert saisie manuelle ou decision par reservation. Lots 4/4bis.</t>
-        </is>
-      </c>
-      <c r="M41" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>MENAGES_EXT||MENAGE_EXTERNE_DATE_ABSENTE</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>MENAGES_EXT</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>MASTER_FACT_MEN_MenagesExternes</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr"/>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>MENAGE_EXTERNE_DATE_ABSENTE</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>9 lignes menages externes sans date_menage precise. Exclues de VUE_ACTIVE.</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr"/>
-      <c r="I42" t="inlineStr"/>
-      <c r="J42" t="inlineStr"/>
-      <c r="K42" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L42" t="inlineStr">
-        <is>
-          <t>Precision date requise aupres du prestataire (Aissata fac.2026-37).</t>
-        </is>
-      </c>
-      <c r="M42" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>2026-02||CLOTURE_IMPOSSIBLE_LIGNE_BANCAIRE_NON_CLASSEE</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>BANQUE</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>BANQUE_LOT8_IMPORT_REF_Cloture</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>2026-02</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>CLOTURE_IMPOSSIBLE_LIGNE_BANCAIRE_NON_CLASSEE</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>Mois 2026-02 statut=OUVERT: 1 lignes RAPPROCHEMENT_REQUIS. Cloture impossible tant que rapprochements non resolus.</t>
-        </is>
-      </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>2026-02</t>
-        </is>
-      </c>
-      <c r="I43" t="inlineStr"/>
-      <c r="J43" t="inlineStr"/>
-      <c r="K43" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L43" t="inlineStr">
-        <is>
-          <t>Exporter donnees Airbnb et rapprocher RAPPROCH_AIRBNB_ATTENTE (Lot 8c).</t>
-        </is>
-      </c>
-      <c r="M43" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>2026-03||CLOTURE_IMPOSSIBLE_LIGNE_BANCAIRE_NON_CLASSEE</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>BANQUE</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>BANQUE_LOT8_IMPORT_REF_Cloture</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>2026-03</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>CLOTURE_IMPOSSIBLE_LIGNE_BANCAIRE_NON_CLASSEE</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>Mois 2026-03 statut=OUVERT: 31 lignes RAPPROCHEMENT_REQUIS. Cloture impossible tant que rapprochements non resolus.</t>
-        </is>
-      </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>2026-03</t>
-        </is>
-      </c>
-      <c r="I44" t="inlineStr"/>
-      <c r="J44" t="inlineStr"/>
-      <c r="K44" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L44" t="inlineStr">
-        <is>
-          <t>Exporter donnees Airbnb et rapprocher RAPPROCH_AIRBNB_ATTENTE (Lot 8c).</t>
-        </is>
-      </c>
-      <c r="M44" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>2026-04||CLOTURE_IMPOSSIBLE_LIGNE_BANCAIRE_NON_CLASSEE</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>BANQUE</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>BANQUE_LOT8_IMPORT_REF_Cloture</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>2026-04</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>CLOTURE_IMPOSSIBLE_LIGNE_BANCAIRE_NON_CLASSEE</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>Mois 2026-04 statut=OUVERT: 20 lignes RAPPROCHEMENT_REQUIS. Cloture impossible tant que rapprochements non resolus.</t>
-        </is>
-      </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>2026-04</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr"/>
-      <c r="J45" t="inlineStr"/>
-      <c r="K45" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L45" t="inlineStr">
-        <is>
-          <t>Exporter donnees Airbnb et rapprocher RAPPROCH_AIRBNB_ATTENTE (Lot 8c).</t>
-        </is>
-      </c>
-      <c r="M45" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
@@ -6094,7 +3564,7 @@
         <v>0</v>
       </c>
       <c r="C5" t="n">
-        <v>41</v>
+        <v>18</v>
       </c>
       <c r="D5" t="n">
         <v>6</v>
@@ -6116,7 +3586,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>41 A_CONTROLER a traiter/valider humainement avant facturation.</t>
+          <t>18 A_CONTROLER a traiter/valider humainement avant facturation.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit fix - AUD-009 date entree gestion en INFO securisee
</commit_message>
<xml_diff>
--- a/02_TRAVAIL/Lot11_Controles/MASTER_CTRL_Coherence.xlsx
+++ b/02_TRAVAIL/Lot11_Controles/MASTER_CTRL_Coherence.xlsx
@@ -736,7 +736,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>A_CONTROLER</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -758,7 +758,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Correction: mettre a jour date_entree_gestion dans REF_Logements (lot separate).</t>
+          <t>INFO justifiee — date_entree_gestion referentielle incoherente, mais calcul forfait securise par D-LOT10-04 via premier mois de flux reel ; REF non modifie, date contractuelle a confirmer si besoin.</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -795,7 +795,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>A_CONTROLER</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -817,7 +817,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Correction: mettre a jour date_entree_gestion dans REF_Logements (lot separate).</t>
+          <t>INFO justifiee — date_entree_gestion referentielle incoherente, mais calcul forfait securise par D-LOT10-04 via premier mois de flux reel ; REF non modifie, date contractuelle a confirmer si besoin.</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -854,7 +854,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>A_CONTROLER</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -876,7 +876,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Correction: mettre a jour date_entree_gestion dans REF_Logements (lot separate).</t>
+          <t>INFO justifiee — date_entree_gestion referentielle incoherente, mais calcul forfait securise par D-LOT10-04 via premier mois de flux reel ; REF non modifie, date contractuelle a confirmer si besoin.</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -913,7 +913,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>A_CONTROLER</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Correction: mettre a jour date_entree_gestion dans REF_Logements (lot separate).</t>
+          <t>INFO justifiee — date_entree_gestion referentielle incoherente, mais calcul forfait securise par D-LOT10-04 via premier mois de flux reel ; REF non modifie, date contractuelle a confirmer si besoin.</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -972,7 +972,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>A_CONTROLER</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -994,7 +994,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Correction: mettre a jour date_entree_gestion dans REF_Logements (lot separate).</t>
+          <t>INFO justifiee — date_entree_gestion referentielle incoherente, mais calcul forfait securise par D-LOT10-04 via premier mois de flux reel ; REF non modifie, date contractuelle a confirmer si besoin.</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1031,7 +1031,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>A_CONTROLER</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1053,7 +1053,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Correction: mettre a jour date_entree_gestion dans REF_Logements (lot separate).</t>
+          <t>INFO justifiee — date_entree_gestion referentielle incoherente, mais calcul forfait securise par D-LOT10-04 via premier mois de flux reel ; REF non modifie, date contractuelle a confirmer si besoin.</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1090,7 +1090,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>A_CONTROLER</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1112,7 +1112,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Correction: mettre a jour date_entree_gestion dans REF_Logements (lot separate).</t>
+          <t>INFO justifiee — date_entree_gestion referentielle incoherente, mais calcul forfait securise par D-LOT10-04 via premier mois de flux reel ; REF non modifie, date contractuelle a confirmer si besoin.</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1149,7 +1149,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>A_CONTROLER</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1171,7 +1171,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>Correction: mettre a jour date_entree_gestion dans REF_Logements (lot separate).</t>
+          <t>INFO justifiee — date_entree_gestion referentielle incoherente, mais calcul forfait securise par D-LOT10-04 via premier mois de flux reel ; REF non modifie, date contractuelle a confirmer si besoin.</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>A_CONTROLER</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1230,7 +1230,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Correction: mettre a jour date_entree_gestion dans REF_Logements (lot separate).</t>
+          <t>INFO justifiee — date_entree_gestion referentielle incoherente, mais calcul forfait securise par D-LOT10-04 via premier mois de flux reel ; REF non modifie, date contractuelle a confirmer si besoin.</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1267,7 +1267,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>A_CONTROLER</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1289,7 +1289,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>Correction: mettre a jour date_entree_gestion dans REF_Logements (lot separate).</t>
+          <t>INFO justifiee — date_entree_gestion referentielle incoherente, mais calcul forfait securise par D-LOT10-04 via premier mois de flux reel ; REF non modifie, date contractuelle a confirmer si besoin.</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -1326,7 +1326,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>A_CONTROLER</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1348,7 +1348,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>Correction: mettre a jour date_entree_gestion dans REF_Logements (lot separate).</t>
+          <t>INFO justifiee — date_entree_gestion referentielle incoherente, mais calcul forfait securise par D-LOT10-04 via premier mois de flux reel ; REF non modifie, date contractuelle a confirmer si besoin.</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -1385,7 +1385,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>A_CONTROLER</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1407,7 +1407,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>Correction: mettre a jour date_entree_gestion dans REF_Logements (lot separate).</t>
+          <t>INFO justifiee — date_entree_gestion referentielle incoherente, mais calcul forfait securise par D-LOT10-04 via premier mois de flux reel ; REF non modifie, date contractuelle a confirmer si besoin.</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -1444,7 +1444,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>A_CONTROLER</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1466,7 +1466,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>Correction: mettre a jour date_entree_gestion dans REF_Logements (lot separate).</t>
+          <t>INFO justifiee — date_entree_gestion referentielle incoherente, mais calcul forfait securise par D-LOT10-04 via premier mois de flux reel ; REF non modifie, date contractuelle a confirmer si besoin.</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -1503,7 +1503,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>A_CONTROLER</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1525,7 +1525,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>Correction: mettre a jour date_entree_gestion dans REF_Logements (lot separate).</t>
+          <t>INFO justifiee — date_entree_gestion referentielle incoherente, mais calcul forfait securise par D-LOT10-04 via premier mois de flux reel ; REF non modifie, date contractuelle a confirmer si besoin.</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -2109,7 +2109,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M22"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2182,7 +2182,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>LOG_0001||CHARGE_FIXE_DATE_ENTREE_GESTION_INCOHERENTE</t>
+          <t>RESERVATIONS||VRBO_MONTANT_NON_RENSEIGNE</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2195,14 +2195,10 @@
           <t>MASTER_CALC_Reservations</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>LOG_0001</t>
-        </is>
-      </c>
+      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>CHARGE_FIXE_DATE_ENTREE_GESTION_INCOHERENTE</t>
+          <t>VRBO_MONTANT_NON_RENSEIGNE</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -2212,15 +2208,11 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Logement LOG_0001: premier mois Flux=2025-07 &lt; date_entree_gestion=2026-01. Utilisation Option A (premier mois Flux) conforme a D-LOT10-04.</t>
+          <t>5 reservations HOSTAWAY_VRBO_A_CONTROLER sans montant valide. Saisie manuelle requise au Lot 4.</t>
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>LOG_0001</t>
-        </is>
-      </c>
+      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
@@ -2229,7 +2221,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Correction: mettre a jour date_entree_gestion dans REF_Logements (lot separate).</t>
+          <t>Lots 4/4bis: saisir montants VRBO dans SAISIE_ReservationsHorsHostaway.xlsx</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -2241,27 +2233,23 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>LOG_0002||CHARGE_FIXE_DATE_ENTREE_GESTION_INCOHERENTE</t>
+          <t>COMMISSIONS||RESERVATION_A_CONTROLER_SANS_COMMISSION</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>RESERVATIONS</t>
+          <t>COMMISSIONS</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>MASTER_CALC_Reservations</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>LOG_0002</t>
-        </is>
-      </c>
+          <t>MASTER_CALC_Commissions</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>CHARGE_FIXE_DATE_ENTREE_GESTION_INCOHERENTE</t>
+          <t>RESERVATION_A_CONTROLER_SANS_COMMISSION</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -2271,15 +2259,11 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Logement LOG_0002: premier mois Flux=2025-02 &lt; date_entree_gestion=2026-01. Utilisation Option A (premier mois Flux) conforme a D-LOT10-04.</t>
+          <t>59 reservations A_CONTROLER exclues du calcul automatique des commissions (VRBO + Direct). Net proprietaire incomplet pour ces 59 reservations.</t>
         </is>
       </c>
       <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>LOG_0002</t>
-        </is>
-      </c>
+      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
@@ -2288,7 +2272,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Correction: mettre a jour date_entree_gestion dans REF_Logements (lot separate).</t>
+          <t>Requiert saisie manuelle ou decision par reservation. Lots 4/4bis.</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -2300,27 +2284,23 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>LOG_0003||CHARGE_FIXE_DATE_ENTREE_GESTION_INCOHERENTE</t>
+          <t>MENAGES_EXT||MENAGE_EXTERNE_ECART_HOSTAWAY</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>RESERVATIONS</t>
+          <t>MENAGES_EXT</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>MASTER_CALC_Reservations</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>LOG_0003</t>
-        </is>
-      </c>
+          <t>VUE_ECART_HOSTAWAY</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>CHARGE_FIXE_DATE_ENTREE_GESTION_INCOHERENTE</t>
+          <t>MENAGE_EXTERNE_ECART_HOSTAWAY</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -2330,15 +2310,11 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Logement LOG_0003: premier mois Flux=2025-02 &lt; date_entree_gestion=2026-01. Utilisation Option A (premier mois Flux) conforme a D-LOT10-04.</t>
+          <t>4 logement(s) avec ecart volume facture vs Hostaway: LOG_0010, LOG_0011, LOG_0013, LOG_0014.</t>
         </is>
       </c>
       <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>LOG_0003</t>
-        </is>
-      </c>
+      <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
@@ -2347,7 +2323,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Correction: mettre a jour date_entree_gestion dans REF_Logements (lot separate).</t>
+          <t>Ecart a valider (interne, hors HA, decalage mois ou saisie). Pas une accusation prestataire.</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -2359,27 +2335,23 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>LOG_0004||CHARGE_FIXE_DATE_ENTREE_GESTION_INCOHERENTE</t>
+          <t>MENAGES_EXT||MENAGE_EXTERNE_LOGEMENT_HORS_HA</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>RESERVATIONS</t>
+          <t>MENAGES_EXT</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>MASTER_CALC_Reservations</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>LOG_0004</t>
-        </is>
-      </c>
+          <t>VUE_ECART_HOSTAWAY</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>CHARGE_FIXE_DATE_ENTREE_GESTION_INCOHERENTE</t>
+          <t>MENAGE_EXTERNE_LOGEMENT_HORS_HA</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -2389,15 +2361,11 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Logement LOG_0004: premier mois Flux=2025-02 &lt; date_entree_gestion=2026-01. Utilisation Option A (premier mois Flux) conforme a D-LOT10-04.</t>
+          <t>2 logement(s) facture(s) absent(s) du comptage Hostaway: LOG_0009, LOG_0016.</t>
         </is>
       </c>
       <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>LOG_0004</t>
-        </is>
-      </c>
+      <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
@@ -2406,7 +2374,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Correction: mettre a jour date_entree_gestion dans REF_Logements (lot separate).</t>
+          <t>Logement archive/hors HA/mapping. A valider, pas une erreur prestataire.</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -2418,27 +2386,27 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>LOG_0006||CHARGE_FIXE_DATE_ENTREE_GESTION_INCOHERENTE</t>
+          <t>2026-02||CLOTURE_IMPOSSIBLE_LIGNE_BANCAIRE_NON_CLASSEE</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>RESERVATIONS</t>
+          <t>BANQUE</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>MASTER_CALC_Reservations</t>
+          <t>BANQUE_LOT8_IMPORT_REF_Cloture</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>LOG_0006</t>
+          <t>2026-02</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>CHARGE_FIXE_DATE_ENTREE_GESTION_INCOHERENTE</t>
+          <t>CLOTURE_IMPOSSIBLE_LIGNE_BANCAIRE_NON_CLASSEE</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -2448,15 +2416,15 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Logement LOG_0006: premier mois Flux=2025-02 &lt; date_entree_gestion=2026-01. Utilisation Option A (premier mois Flux) conforme a D-LOT10-04.</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>LOG_0006</t>
-        </is>
-      </c>
+          <t>Mois 2026-02 statut=OUVERT: 1 lignes RAPPROCHEMENT_REQUIS. Cloture impossible tant que rapprochements non resolus.</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>2026-02</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
@@ -2465,7 +2433,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Correction: mettre a jour date_entree_gestion dans REF_Logements (lot separate).</t>
+          <t>Exporter donnees Airbnb et rapprocher RAPPROCH_AIRBNB_ATTENTE (Lot 8c).</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -2477,27 +2445,27 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>LOG_0007||CHARGE_FIXE_DATE_ENTREE_GESTION_INCOHERENTE</t>
+          <t>2026-03||CLOTURE_IMPOSSIBLE_LIGNE_BANCAIRE_NON_CLASSEE</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>RESERVATIONS</t>
+          <t>BANQUE</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>MASTER_CALC_Reservations</t>
+          <t>BANQUE_LOT8_IMPORT_REF_Cloture</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>LOG_0007</t>
+          <t>2026-03</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>CHARGE_FIXE_DATE_ENTREE_GESTION_INCOHERENTE</t>
+          <t>CLOTURE_IMPOSSIBLE_LIGNE_BANCAIRE_NON_CLASSEE</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -2507,15 +2475,15 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Logement LOG_0007: premier mois Flux=2025-03 &lt; date_entree_gestion=2026-01. Utilisation Option A (premier mois Flux) conforme a D-LOT10-04.</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>LOG_0007</t>
-        </is>
-      </c>
+          <t>Mois 2026-03 statut=OUVERT: 31 lignes RAPPROCHEMENT_REQUIS. Cloture impossible tant que rapprochements non resolus.</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
@@ -2524,7 +2492,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Correction: mettre a jour date_entree_gestion dans REF_Logements (lot separate).</t>
+          <t>Exporter donnees Airbnb et rapprocher RAPPROCH_AIRBNB_ATTENTE (Lot 8c).</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -2536,27 +2504,27 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>LOG_0008||CHARGE_FIXE_DATE_ENTREE_GESTION_INCOHERENTE</t>
+          <t>2026-04||CLOTURE_IMPOSSIBLE_LIGNE_BANCAIRE_NON_CLASSEE</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>RESERVATIONS</t>
+          <t>BANQUE</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>MASTER_CALC_Reservations</t>
+          <t>BANQUE_LOT8_IMPORT_REF_Cloture</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>LOG_0008</t>
+          <t>2026-04</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>CHARGE_FIXE_DATE_ENTREE_GESTION_INCOHERENTE</t>
+          <t>CLOTURE_IMPOSSIBLE_LIGNE_BANCAIRE_NON_CLASSEE</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -2566,15 +2534,15 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Logement LOG_0008: premier mois Flux=2025-02 &lt; date_entree_gestion=2026-01. Utilisation Option A (premier mois Flux) conforme a D-LOT10-04.</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>LOG_0008</t>
-        </is>
-      </c>
+          <t>Mois 2026-04 statut=OUVERT: 20 lignes RAPPROCHEMENT_REQUIS. Cloture impossible tant que rapprochements non resolus.</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
@@ -2583,804 +2551,10 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Correction: mettre a jour date_entree_gestion dans REF_Logements (lot separate).</t>
+          <t>Exporter donnees Airbnb et rapprocher RAPPROCH_AIRBNB_ATTENTE (Lot 8c).</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
-        <is>
-          <t>2026-06-18</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>LOG_0010||CHARGE_FIXE_DATE_ENTREE_GESTION_INCOHERENTE</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>RESERVATIONS</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>MASTER_CALC_Reservations</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>LOG_0010</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>CHARGE_FIXE_DATE_ENTREE_GESTION_INCOHERENTE</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>Logement LOG_0010: premier mois Flux=2025-01 &lt; date_entree_gestion=2026-01. Utilisation Option A (premier mois Flux) conforme a D-LOT10-04.</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>LOG_0010</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>Correction: mettre a jour date_entree_gestion dans REF_Logements (lot separate).</t>
-        </is>
-      </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>2026-06-18</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>LOG_0011||CHARGE_FIXE_DATE_ENTREE_GESTION_INCOHERENTE</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>RESERVATIONS</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>MASTER_CALC_Reservations</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>LOG_0011</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>CHARGE_FIXE_DATE_ENTREE_GESTION_INCOHERENTE</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Logement LOG_0011: premier mois Flux=2025-01 &lt; date_entree_gestion=2026-01. Utilisation Option A (premier mois Flux) conforme a D-LOT10-04.</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>LOG_0011</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>Correction: mettre a jour date_entree_gestion dans REF_Logements (lot separate).</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>2026-06-18</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>LOG_0012||CHARGE_FIXE_DATE_ENTREE_GESTION_INCOHERENTE</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>RESERVATIONS</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>MASTER_CALC_Reservations</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>LOG_0012</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>CHARGE_FIXE_DATE_ENTREE_GESTION_INCOHERENTE</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>Logement LOG_0012: premier mois Flux=2025-02 &lt; date_entree_gestion=2026-01. Utilisation Option A (premier mois Flux) conforme a D-LOT10-04.</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>LOG_0012</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>Correction: mettre a jour date_entree_gestion dans REF_Logements (lot separate).</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>2026-06-18</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>LOG_0013||CHARGE_FIXE_DATE_ENTREE_GESTION_INCOHERENTE</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>RESERVATIONS</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>MASTER_CALC_Reservations</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>LOG_0013</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>CHARGE_FIXE_DATE_ENTREE_GESTION_INCOHERENTE</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>Logement LOG_0013: premier mois Flux=2025-01 &lt; date_entree_gestion=2026-01. Utilisation Option A (premier mois Flux) conforme a D-LOT10-04.</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>LOG_0013</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>Correction: mettre a jour date_entree_gestion dans REF_Logements (lot separate).</t>
-        </is>
-      </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>2026-06-18</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>LOG_0014||CHARGE_FIXE_DATE_ENTREE_GESTION_INCOHERENTE</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>RESERVATIONS</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>MASTER_CALC_Reservations</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>LOG_0014</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>CHARGE_FIXE_DATE_ENTREE_GESTION_INCOHERENTE</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Logement LOG_0014: premier mois Flux=2025-01 &lt; date_entree_gestion=2026-01. Utilisation Option A (premier mois Flux) conforme a D-LOT10-04.</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>LOG_0014</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>Correction: mettre a jour date_entree_gestion dans REF_Logements (lot separate).</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>2026-06-18</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>LOG_0015||CHARGE_FIXE_DATE_ENTREE_GESTION_INCOHERENTE</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>RESERVATIONS</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>MASTER_CALC_Reservations</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>LOG_0015</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>CHARGE_FIXE_DATE_ENTREE_GESTION_INCOHERENTE</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>Logement LOG_0015: premier mois Flux=2025-02 &lt; date_entree_gestion=2026-01. Utilisation Option A (premier mois Flux) conforme a D-LOT10-04.</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>LOG_0015</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>Correction: mettre a jour date_entree_gestion dans REF_Logements (lot separate).</t>
-        </is>
-      </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>2026-06-18</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>LOG_0016||CHARGE_FIXE_DATE_ENTREE_GESTION_INCOHERENTE</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>RESERVATIONS</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>MASTER_CALC_Reservations</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>LOG_0016</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>CHARGE_FIXE_DATE_ENTREE_GESTION_INCOHERENTE</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>Logement LOG_0016: premier mois Flux=2025-05 &lt; date_entree_gestion=2026-01. Utilisation Option A (premier mois Flux) conforme a D-LOT10-04.</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>LOG_0016</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>Correction: mettre a jour date_entree_gestion dans REF_Logements (lot separate).</t>
-        </is>
-      </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>2026-06-18</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>RESERVATIONS||VRBO_MONTANT_NON_RENSEIGNE</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>RESERVATIONS</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>MASTER_CALC_Reservations</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>VRBO_MONTANT_NON_RENSEIGNE</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>5 reservations HOSTAWAY_VRBO_A_CONTROLER sans montant valide. Saisie manuelle requise au Lot 4.</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>Lots 4/4bis: saisir montants VRBO dans SAISIE_ReservationsHorsHostaway.xlsx</t>
-        </is>
-      </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>2026-06-18</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>COMMISSIONS||RESERVATION_A_CONTROLER_SANS_COMMISSION</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>COMMISSIONS</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>MASTER_CALC_Commissions</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>RESERVATION_A_CONTROLER_SANS_COMMISSION</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>59 reservations A_CONTROLER exclues du calcul automatique des commissions (VRBO + Direct). Net proprietaire incomplet pour ces 59 reservations.</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>Requiert saisie manuelle ou decision par reservation. Lots 4/4bis.</t>
-        </is>
-      </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>2026-06-18</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>MENAGES_EXT||MENAGE_EXTERNE_ECART_HOSTAWAY</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>MENAGES_EXT</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>VUE_ECART_HOSTAWAY</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>MENAGE_EXTERNE_ECART_HOSTAWAY</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>4 logement(s) avec ecart volume facture vs Hostaway: LOG_0010, LOG_0011, LOG_0013, LOG_0014.</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>Ecart a valider (interne, hors HA, decalage mois ou saisie). Pas une accusation prestataire.</t>
-        </is>
-      </c>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>2026-06-18</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>MENAGES_EXT||MENAGE_EXTERNE_LOGEMENT_HORS_HA</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>MENAGES_EXT</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>VUE_ECART_HOSTAWAY</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>MENAGE_EXTERNE_LOGEMENT_HORS_HA</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>2 logement(s) facture(s) absent(s) du comptage Hostaway: LOG_0009, LOG_0016.</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>Logement archive/hors HA/mapping. A valider, pas une erreur prestataire.</t>
-        </is>
-      </c>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>2026-06-18</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>2026-02||CLOTURE_IMPOSSIBLE_LIGNE_BANCAIRE_NON_CLASSEE</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>BANQUE</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>BANQUE_LOT8_IMPORT_REF_Cloture</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>2026-02</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>CLOTURE_IMPOSSIBLE_LIGNE_BANCAIRE_NON_CLASSEE</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>Mois 2026-02 statut=OUVERT: 1 lignes RAPPROCHEMENT_REQUIS. Cloture impossible tant que rapprochements non resolus.</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>2026-02</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>Exporter donnees Airbnb et rapprocher RAPPROCH_AIRBNB_ATTENTE (Lot 8c).</t>
-        </is>
-      </c>
-      <c r="M20" t="inlineStr">
-        <is>
-          <t>2026-06-18</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>2026-03||CLOTURE_IMPOSSIBLE_LIGNE_BANCAIRE_NON_CLASSEE</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>BANQUE</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>BANQUE_LOT8_IMPORT_REF_Cloture</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>2026-03</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>CLOTURE_IMPOSSIBLE_LIGNE_BANCAIRE_NON_CLASSEE</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>Mois 2026-03 statut=OUVERT: 31 lignes RAPPROCHEMENT_REQUIS. Cloture impossible tant que rapprochements non resolus.</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>2026-03</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>Exporter donnees Airbnb et rapprocher RAPPROCH_AIRBNB_ATTENTE (Lot 8c).</t>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>2026-06-18</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>2026-04||CLOTURE_IMPOSSIBLE_LIGNE_BANCAIRE_NON_CLASSEE</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>BANQUE</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>BANQUE_LOT8_IMPORT_REF_Cloture</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>2026-04</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>CLOTURE_IMPOSSIBLE_LIGNE_BANCAIRE_NON_CLASSEE</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>A_CONTROLER</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>Mois 2026-04 statut=OUVERT: 20 lignes RAPPROCHEMENT_REQUIS. Cloture impossible tant que rapprochements non resolus.</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>2026-04</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>OUVERT</t>
-        </is>
-      </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>Exporter donnees Airbnb et rapprocher RAPPROCH_AIRBNB_ATTENTE (Lot 8c).</t>
-        </is>
-      </c>
-      <c r="M22" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
@@ -3560,10 +2734,10 @@
         <v>0</v>
       </c>
       <c r="C5" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="D5" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -3582,7 +2756,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>18 A_CONTROLER a traiter/valider humainement avant facturation.</t>
+          <t>4 A_CONTROLER a traiter/valider humainement avant facturation.</t>
         </is>
       </c>
     </row>

</xml_diff>